<commit_message>
Cierre de hilos: cohorte 5 oct (8-12 AM super / 6:30-8:30 PM intensivo, 17+, minimo 6, jornada la define el cliente no se empuja), separacion unificada \$300k en kit/tarjeta/guia/motor/bot, vigencia se CUMPLE, bot con datos confirmados, motor v3 con hoja Arranque en repo
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7C5dx3NvDfXiv3CfhPMa
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/MOTOR_CUOTAS_FONDO_2026.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/MOTOR_CUOTAS_FONDO_2026.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A2-B2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B1-B2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solo B2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARRANQUE A1+A2" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,7 +503,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reserva $100-150 mil dia 1 -&gt; cuota inicial max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
+          <t>Separacion de cupo $300.000 (se cruza con la inicial) -&gt; cuota inicial min 20% max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1343,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reserva $100-150 mil dia 1 -&gt; cuota inicial max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
+          <t>Separacion de cupo $300.000 (se cruza con la inicial) -&gt; cuota inicial min 20% max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2183,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reserva $100-150 mil dia 1 -&gt; cuota inicial max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
+          <t>Separacion de cupo $300.000 (se cruza con la inicial) -&gt; cuota inicial min 20% max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2870,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Reserva $100-150 mil dia 1 -&gt; cuota inicial max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
+          <t>Separacion de cupo $300.000 (se cruza con la inicial) -&gt; cuota inicial min 20% max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
         </is>
       </c>
     </row>
@@ -3266,4 +3267,160 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HEIIU - MOTOR DE CUOTAS 2026 - USO INTERNO (jamas mostrar al cliente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ARRANQUE A1+A2 - PRECIO UNICO DE LANZAMIENTO: $2.990.000 (200 horas) - SIN BECAS - Interes credito directo: 1,9% mensual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>REGLA: se termina de pagar antes de terminar. Super intensivo 20h/sem ~2,5 meses: MAX 2 CUOTAS. Intensivo 10h/sem ~5 meses: MAX 4 CUOTAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Separacion de cupo $300.000 (se cruza con la inicial) -&gt; cuota inicial min 20% max 3 dias -&gt; cuotas desde dia 30. Credito SIEMPRE con pagare + carta + plan de pagos firmados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>PRECIO (contado o a cuotas): $2.990.000</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Cuota inicial</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>2 cuotas</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>3 cuotas</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>4 cuotas</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>20% = $598.000</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>1230193</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>827822</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>626672</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Super intensivo: solo columna 2 cuotas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>30% = $897.000</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>1076419</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>724344</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>548338</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>40% = $1.196.000</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>922645</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>620867</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>470004</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>50% = $1.495.000</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>768871</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>517389</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>391670</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Motor de cuotas: rotulo de Transformacion incluye al afiliado a Cajasan; Arranque sin beca tambien para afiliados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/MOTOR_CUOTAS_FONDO_2026.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/MOTOR_CUOTAS_FONDO_2026.xlsx
@@ -507,10 +507,11 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TRANSFORMACION  -  Beca del Fondo: contado 45% / cuotas 36%</t>
+          <t>TRANSFORMACION (estrato 1-2 con soporte O AFILIADO A CAJASAN con carne)  -  Beca del Fondo: contado 45% / cuotas 36%</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -770,6 +771,7 @@
         <v>282718</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -1033,6 +1035,7 @@
         <v>328659</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -1347,10 +1350,11 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TRANSFORMACION  -  Beca del Fondo: contado 36% / cuotas 27%</t>
+          <t>TRANSFORMACION (estrato 1-2 con soporte O AFILIADO A CAJASAN con carne)  -  Beca del Fondo: contado 36% / cuotas 27%</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -1610,6 +1614,7 @@
         <v>263290</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -1873,6 +1878,7 @@
         <v>291423</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -2187,10 +2193,11 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TRANSFORMACION  -  Beca del Fondo: contado 24.8% / cuotas 15.8%</t>
+          <t>TRANSFORMACION (estrato 1-2 con soporte O AFILIADO A CAJASAN con carne)  -  Beca del Fondo: contado 24.8% / cuotas 15.8%</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -2399,6 +2406,7 @@
         <v>296702</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -2611,6 +2619,7 @@
         <v>312912</v>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
@@ -2874,10 +2883,11 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TRANSFORMACION  -  Beca del Fondo: contado 20.3% / cuotas 11.3%</t>
+          <t>TRANSFORMACION (estrato 1-2 con soporte O AFILIADO A CAJASAN con carne)  -  Beca del Fondo: contado 20.3% / cuotas 11.3%</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -3004,6 +3014,7 @@
         <v>272236</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
@@ -3134,6 +3145,7 @@
         <v>282364</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -3295,7 +3307,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ARRANQUE A1+A2 - PRECIO UNICO DE LANZAMIENTO: $2.990.000 (200 horas) - SIN BECAS - Interes credito directo: 1,9% mensual</t>
+          <t>ARRANQUE A1+A2 - PRECIO UNICO DE LANZAMIENTO: $2.990.000 (200 horas) - SIN BECAS - Interes credito directo: 1,9% mensual - Afiliado Cajasan: mismo precio, sin beca</t>
         </is>
       </c>
     </row>
@@ -3313,6 +3325,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>

</xml_diff>